<commit_message>
Added new bugs to fix later...
</commit_message>
<xml_diff>
--- a/assets/2--Morning Shift Stands Data.xlsx
+++ b/assets/2--Morning Shift Stands Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ruhan\School Bus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ruhan\School Bus\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56FBA1C-CB14-41C3-846E-CB7214BB5FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33DF3ED-20FF-4F8A-8D4C-A90A92F1460B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -251,7 +251,7 @@
     <t>C &amp; B</t>
   </si>
   <si>
-    <t>First Row can not be readed (standName-number-routeName)</t>
+    <t>First Row can not be readed (standName-studentNumber)</t>
   </si>
 </sst>
 </file>
@@ -289,13 +289,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -605,630 +604,630 @@
   <dimension ref="A1:C73"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.77734375" style="2"/>
-    <col min="3" max="3" width="23.109375" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.77734375" style="2"/>
+    <col min="1" max="1" width="25.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.77734375" style="1"/>
+    <col min="3" max="3" width="23.109375" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>9</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>32</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>14</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>10</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>14</v>
       </c>
-      <c r="C14" s="3"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>39</v>
       </c>
-      <c r="C17" s="3"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>23</v>
       </c>
-      <c r="C23" s="3"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>63</v>
       </c>
-      <c r="C24" s="3"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="1">
         <v>9</v>
       </c>
-      <c r="C25" s="3"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="1">
         <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="1">
         <v>7</v>
       </c>
-      <c r="C28" s="3"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="1">
         <v>2</v>
       </c>
-      <c r="C29" s="3"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="1">
         <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="1">
         <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="1">
         <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="1">
         <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="1">
         <v>23</v>
       </c>
-      <c r="C34" s="3"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="1">
         <v>13</v>
       </c>
-      <c r="C35" s="3"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36" s="1">
         <v>30</v>
       </c>
-      <c r="C36" s="3"/>
+      <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="1">
         <v>13</v>
       </c>
-      <c r="C37" s="3"/>
+      <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="1">
         <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="1">
         <v>6</v>
       </c>
-      <c r="C39" s="3"/>
+      <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="1">
         <v>19</v>
       </c>
-      <c r="C40" s="3"/>
+      <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="1">
         <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="1">
         <v>7</v>
       </c>
-      <c r="C42" s="3"/>
+      <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="1">
         <v>34</v>
       </c>
-      <c r="C43" s="3"/>
+      <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="1">
         <v>1</v>
       </c>
-      <c r="C44" s="3"/>
+      <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="1">
         <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="1">
         <v>8</v>
       </c>
-      <c r="C46" s="3"/>
+      <c r="C46" s="2"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="1">
         <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="1">
         <v>5</v>
       </c>
-      <c r="C48" s="3"/>
+      <c r="C48" s="2"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="1">
         <v>4</v>
       </c>
-      <c r="C49" s="3"/>
+      <c r="C49" s="2"/>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
+      <c r="A50" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="1">
         <v>7</v>
       </c>
-      <c r="C50" s="3"/>
+      <c r="C50" s="2"/>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="1">
         <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
+      <c r="A52" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="1">
         <v>12</v>
       </c>
-      <c r="C52" s="3"/>
+      <c r="C52" s="2"/>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
+      <c r="A53" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="1">
         <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
+      <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="1">
         <v>57</v>
       </c>
-      <c r="C54" s="3"/>
+      <c r="C54" s="2"/>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
+      <c r="A55" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="1">
         <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="1">
         <v>8</v>
       </c>
-      <c r="C56" s="3"/>
+      <c r="C56" s="2"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
+      <c r="A57" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="2" t="s">
+      <c r="A59" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="1">
         <v>9</v>
       </c>
-      <c r="C59" s="3"/>
+      <c r="C59" s="2"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="1">
         <v>16</v>
       </c>
-      <c r="C60" s="3"/>
+      <c r="C60" s="2"/>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="1">
         <v>15</v>
       </c>
-      <c r="C61" s="3"/>
+      <c r="C61" s="2"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="1">
         <v>19</v>
       </c>
-      <c r="C62" s="3"/>
+      <c r="C62" s="2"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
+      <c r="A63" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="1">
         <v>31</v>
       </c>
-      <c r="C63" s="3"/>
+      <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
+      <c r="A64" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="1">
         <v>4</v>
       </c>
-      <c r="C64" s="3"/>
+      <c r="C64" s="2"/>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="1">
         <v>91</v>
       </c>
-      <c r="C65" s="3"/>
+      <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
+      <c r="A66" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="1">
         <v>24</v>
       </c>
-      <c r="C66" s="3"/>
+      <c r="C66" s="2"/>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
+      <c r="A67" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="1">
         <v>23</v>
       </c>
-      <c r="C67" s="3"/>
+      <c r="C67" s="2"/>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
+      <c r="A68" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="1">
         <v>15</v>
       </c>
-      <c r="C68" s="3"/>
+      <c r="C68" s="2"/>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="2" t="s">
+      <c r="A69" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="2" t="s">
+      <c r="A70" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="1">
         <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="2" t="s">
+      <c r="A71" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="1">
         <v>2</v>
       </c>
-      <c r="C71" s="3"/>
+      <c r="C71" s="2"/>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="2" t="s">
+      <c r="A72" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="1">
         <v>11</v>
       </c>
-      <c r="C72" s="3"/>
+      <c r="C72" s="2"/>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
+      <c r="A73" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="1">
         <v>25</v>
       </c>
     </row>

</xml_diff>